<commit_message>
vault backup: 2026-03-25 10:14:47
</commit_message>
<xml_diff>
--- a/开发平台/codex/项目/人员简历筛选和重组/output/spreadsheet/风险项目完整清单_v1.2.xlsx
+++ b/开发平台/codex/项目/人员简历筛选和重组/output/spreadsheet/风险项目完整清单_v1.2.xlsx
@@ -462,7 +462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E88"/>
+  <dimension ref="A1:G88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -470,6 +470,7 @@
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -479,6 +480,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -503,6 +505,11 @@
       <c r="E3" s="2" t="inlineStr">
         <is>
           <t>客户要求年限</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>是否达标</t>
         </is>
       </c>
     </row>
@@ -526,6 +533,11 @@
       <c r="E4" s="5" t="n">
         <v>5</v>
       </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="n">
@@ -547,6 +559,11 @@
       <c r="E5" s="5" t="n">
         <v>5</v>
       </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="n">
@@ -568,6 +585,11 @@
       <c r="E6" s="5" t="n">
         <v>3</v>
       </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="n">
@@ -589,6 +611,11 @@
       <c r="E7" s="5" t="n">
         <v>3</v>
       </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="n">
@@ -609,6 +636,11 @@
       </c>
       <c r="E8" s="5" t="n">
         <v>0</v>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
       </c>
     </row>
     <row r="9">
@@ -631,6 +663,11 @@
       <c r="E9" s="5" t="n">
         <v>5</v>
       </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="n">
@@ -652,6 +689,11 @@
       <c r="E10" s="5" t="n">
         <v>3</v>
       </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="n">
@@ -673,6 +715,11 @@
       <c r="E11" s="5" t="n">
         <v>3</v>
       </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="n">
@@ -694,6 +741,11 @@
       <c r="E12" s="5" t="n">
         <v>5</v>
       </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="n">
@@ -715,6 +767,11 @@
       <c r="E13" s="5" t="n">
         <v>5</v>
       </c>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="n">
@@ -736,6 +793,11 @@
       <c r="E14" s="5" t="n">
         <v>3</v>
       </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="n">
@@ -757,6 +819,11 @@
       <c r="E15" s="5" t="n">
         <v>5</v>
       </c>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="n">
@@ -778,6 +845,11 @@
       <c r="E16" s="5" t="n">
         <v>3</v>
       </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="n">
@@ -799,6 +871,11 @@
       <c r="E17" s="5" t="n">
         <v>5</v>
       </c>
+      <c r="F17" s="5" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="n">
@@ -820,6 +897,11 @@
       <c r="E18" s="5" t="n">
         <v>3</v>
       </c>
+      <c r="F18" s="5" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="n">
@@ -841,6 +923,11 @@
       <c r="E19" s="5" t="n">
         <v>0</v>
       </c>
+      <c r="F19" s="5" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="n">
@@ -862,6 +949,11 @@
       <c r="E20" s="5" t="n">
         <v>5</v>
       </c>
+      <c r="F20" s="5" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="n">
@@ -883,6 +975,11 @@
       <c r="E21" s="5" t="n">
         <v>3</v>
       </c>
+      <c r="F21" s="5" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="n">
@@ -904,6 +1001,11 @@
       <c r="E22" s="5" t="n">
         <v>5</v>
       </c>
+      <c r="F22" s="5" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="n">
@@ -925,6 +1027,11 @@
       <c r="E23" s="5" t="n">
         <v>5</v>
       </c>
+      <c r="F23" s="5" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="n">
@@ -946,6 +1053,11 @@
       <c r="E24" s="5" t="n">
         <v>3</v>
       </c>
+      <c r="F24" s="5" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="n">
@@ -967,6 +1079,11 @@
       <c r="E25" s="5" t="n">
         <v>3</v>
       </c>
+      <c r="F25" s="5" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="n">
@@ -988,6 +1105,11 @@
       <c r="E26" s="5" t="n">
         <v>0</v>
       </c>
+      <c r="F26" s="5" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="n">
@@ -1009,6 +1131,11 @@
       <c r="E27" s="5" t="n">
         <v>0</v>
       </c>
+      <c r="F27" s="5" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="n">
@@ -1030,6 +1157,11 @@
       <c r="E28" s="5" t="n">
         <v>5</v>
       </c>
+      <c r="F28" s="5" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="n">
@@ -1051,6 +1183,11 @@
       <c r="E29" s="5" t="n">
         <v>5</v>
       </c>
+      <c r="F29" s="5" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="3" t="n">
@@ -1072,6 +1209,11 @@
       <c r="E30" s="5" t="n">
         <v>3</v>
       </c>
+      <c r="F30" s="5" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="n">
@@ -1093,6 +1235,11 @@
       <c r="E31" s="5" t="n">
         <v>0</v>
       </c>
+      <c r="F31" s="5" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="3" t="n">
@@ -1114,6 +1261,11 @@
       <c r="E32" s="5" t="n">
         <v>3</v>
       </c>
+      <c r="F32" s="5" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="n">
@@ -1135,6 +1287,11 @@
       <c r="E33" s="5" t="n">
         <v>0</v>
       </c>
+      <c r="F33" s="5" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="3" t="n">
@@ -1156,6 +1313,11 @@
       <c r="E34" s="5" t="n">
         <v>5</v>
       </c>
+      <c r="F34" s="5" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="n">
@@ -1177,6 +1339,11 @@
       <c r="E35" s="5" t="n">
         <v>3</v>
       </c>
+      <c r="F35" s="5" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="3" t="n">
@@ -1198,6 +1365,11 @@
       <c r="E36" s="5" t="n">
         <v>3</v>
       </c>
+      <c r="F36" s="5" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="3" t="n">
@@ -1219,6 +1391,11 @@
       <c r="E37" s="5" t="n">
         <v>5</v>
       </c>
+      <c r="F37" s="5" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="3" t="n">
@@ -1240,6 +1417,11 @@
       <c r="E38" s="5" t="n">
         <v>5</v>
       </c>
+      <c r="F38" s="5" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="3" t="n">
@@ -1261,6 +1443,11 @@
       <c r="E39" s="5" t="n">
         <v>3</v>
       </c>
+      <c r="F39" s="5" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="3" t="n">
@@ -1282,6 +1469,11 @@
       <c r="E40" s="5" t="n">
         <v>5</v>
       </c>
+      <c r="F40" s="5" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="3" t="n">
@@ -1303,6 +1495,11 @@
       <c r="E41" s="5" t="n">
         <v>3</v>
       </c>
+      <c r="F41" s="5" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="3" t="n">
@@ -1324,6 +1521,11 @@
       <c r="E42" s="5" t="n">
         <v>0</v>
       </c>
+      <c r="F42" s="5" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="3" t="n">
@@ -1345,6 +1547,11 @@
       <c r="E43" s="5" t="n">
         <v>3</v>
       </c>
+      <c r="F43" s="5" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="3" t="n">
@@ -1366,6 +1573,11 @@
       <c r="E44" s="5" t="n">
         <v>0</v>
       </c>
+      <c r="F44" s="5" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="3" t="n">
@@ -1387,6 +1599,11 @@
       <c r="E45" s="5" t="n">
         <v>5</v>
       </c>
+      <c r="F45" s="5" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="3" t="n">
@@ -1408,6 +1625,11 @@
       <c r="E46" s="5" t="n">
         <v>5</v>
       </c>
+      <c r="F46" s="5" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="3" t="n">
@@ -1429,6 +1651,11 @@
       <c r="E47" s="5" t="n">
         <v>3</v>
       </c>
+      <c r="F47" s="5" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="3" t="n">
@@ -1450,6 +1677,11 @@
       <c r="E48" s="5" t="n">
         <v>3</v>
       </c>
+      <c r="F48" s="5" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="3" t="n">
@@ -1471,6 +1703,11 @@
       <c r="E49" s="5" t="n">
         <v>0</v>
       </c>
+      <c r="F49" s="5" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="3" t="n">
@@ -1492,6 +1729,11 @@
       <c r="E50" s="5" t="n">
         <v>0</v>
       </c>
+      <c r="F50" s="5" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="3" t="n">
@@ -1513,6 +1755,11 @@
       <c r="E51" s="5" t="n">
         <v>5</v>
       </c>
+      <c r="F51" s="5" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="3" t="n">
@@ -1534,6 +1781,11 @@
       <c r="E52" s="5" t="n">
         <v>5</v>
       </c>
+      <c r="F52" s="5" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="3" t="n">
@@ -1555,6 +1807,11 @@
       <c r="E53" s="5" t="n">
         <v>3</v>
       </c>
+      <c r="F53" s="5" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="3" t="n">
@@ -1576,6 +1833,11 @@
       <c r="E54" s="5" t="n">
         <v>15</v>
       </c>
+      <c r="F54" s="5" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="3" t="n">
@@ -1597,6 +1859,11 @@
       <c r="E55" s="5" t="n">
         <v>15</v>
       </c>
+      <c r="F55" s="5" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="3" t="n">
@@ -1615,7 +1882,14 @@
       <c r="D56" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="E56" s="5" t="n"/>
+      <c r="E56" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="F56" s="5" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="3" t="n">
@@ -1634,7 +1908,14 @@
       <c r="D57" s="5" t="n">
         <v>6.7</v>
       </c>
-      <c r="E57" s="5" t="n"/>
+      <c r="E57" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="F57" s="5" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="3" t="n">
@@ -1653,7 +1934,14 @@
       <c r="D58" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="E58" s="5" t="n"/>
+      <c r="E58" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="F58" s="5" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="3" t="n">
@@ -1672,7 +1960,14 @@
       <c r="D59" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="E59" s="5" t="n"/>
+      <c r="E59" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F59" s="5" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="3" t="n">
@@ -1691,7 +1986,14 @@
       <c r="D60" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="E60" s="5" t="n"/>
+      <c r="E60" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F60" s="5" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="3" t="n">
@@ -1710,7 +2012,14 @@
       <c r="D61" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="E61" s="5" t="n"/>
+      <c r="E61" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F61" s="5" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="3" t="n">
@@ -1729,7 +2038,14 @@
       <c r="D62" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="E62" s="5" t="n"/>
+      <c r="E62" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F62" s="5" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="3" t="n">
@@ -1748,7 +2064,14 @@
       <c r="D63" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="E63" s="5" t="n"/>
+      <c r="E63" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F63" s="5" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="3" t="n">
@@ -1767,7 +2090,14 @@
       <c r="D64" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="E64" s="5" t="n"/>
+      <c r="E64" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F64" s="5" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="3" t="n">
@@ -1786,7 +2116,14 @@
       <c r="D65" s="5" t="n">
         <v>0.3</v>
       </c>
-      <c r="E65" s="5" t="n"/>
+      <c r="E65" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F65" s="5" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="3" t="n">
@@ -1808,6 +2145,11 @@
       <c r="E66" s="5" t="n">
         <v>5</v>
       </c>
+      <c r="F66" s="5" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="3" t="n">
@@ -1829,6 +2171,11 @@
       <c r="E67" s="5" t="n">
         <v>5</v>
       </c>
+      <c r="F67" s="5" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="3" t="n">
@@ -1850,6 +2197,11 @@
       <c r="E68" s="5" t="n">
         <v>5</v>
       </c>
+      <c r="F68" s="5" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="3" t="n">
@@ -1871,6 +2223,11 @@
       <c r="E69" s="5" t="n">
         <v>5</v>
       </c>
+      <c r="F69" s="5" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="3" t="n">
@@ -1892,6 +2249,11 @@
       <c r="E70" s="5" t="n">
         <v>5</v>
       </c>
+      <c r="F70" s="5" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="3" t="n">
@@ -1913,6 +2275,11 @@
       <c r="E71" s="5" t="n">
         <v>5</v>
       </c>
+      <c r="F71" s="5" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="3" t="n">
@@ -1934,6 +2301,11 @@
       <c r="E72" s="5" t="n">
         <v>7</v>
       </c>
+      <c r="F72" s="5" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="3" t="n">
@@ -1955,6 +2327,11 @@
       <c r="E73" s="5" t="n">
         <v>5</v>
       </c>
+      <c r="F73" s="5" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="3" t="n">
@@ -1976,6 +2353,11 @@
       <c r="E74" s="5" t="n">
         <v>5</v>
       </c>
+      <c r="F74" s="5" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="3" t="n">
@@ -1997,6 +2379,11 @@
       <c r="E75" s="5" t="n">
         <v>5</v>
       </c>
+      <c r="F75" s="5" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="3" t="n">
@@ -2018,6 +2405,11 @@
       <c r="E76" s="5" t="n">
         <v>3</v>
       </c>
+      <c r="F76" s="5" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="3" t="n">
@@ -2039,6 +2431,11 @@
       <c r="E77" s="5" t="n">
         <v>5</v>
       </c>
+      <c r="F77" s="5" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="3" t="n">
@@ -2060,6 +2457,11 @@
       <c r="E78" s="5" t="n">
         <v>0</v>
       </c>
+      <c r="F78" s="5" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="3" t="n">
@@ -2081,6 +2483,11 @@
       <c r="E79" s="5" t="n">
         <v>3</v>
       </c>
+      <c r="F79" s="5" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="3" t="n">
@@ -2102,6 +2509,11 @@
       <c r="E80" s="5" t="n">
         <v>3</v>
       </c>
+      <c r="F80" s="5" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="3" t="n">
@@ -2123,6 +2535,11 @@
       <c r="E81" s="5" t="n">
         <v>5</v>
       </c>
+      <c r="F81" s="5" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="3" t="n">
@@ -2144,6 +2561,11 @@
       <c r="E82" s="5" t="n">
         <v>3</v>
       </c>
+      <c r="F82" s="5" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="3" t="n">
@@ -2165,6 +2587,11 @@
       <c r="E83" s="5" t="n">
         <v>5</v>
       </c>
+      <c r="F83" s="5" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="3" t="n">
@@ -2186,6 +2613,11 @@
       <c r="E84" s="5" t="n">
         <v>0</v>
       </c>
+      <c r="F84" s="5" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="3" t="n">
@@ -2207,6 +2639,11 @@
       <c r="E85" s="5" t="n">
         <v>5</v>
       </c>
+      <c r="F85" s="5" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="3" t="n">
@@ -2228,6 +2665,11 @@
       <c r="E86" s="5" t="n">
         <v>3</v>
       </c>
+      <c r="F86" s="5" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="3" t="n">
@@ -2249,6 +2691,11 @@
       <c r="E87" s="5" t="n">
         <v>5</v>
       </c>
+      <c r="F87" s="5" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="3" t="n">
@@ -2270,10 +2717,15 @@
       <c r="E88" s="5" t="n">
         <v>3</v>
       </c>
+      <c r="F88" s="5" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A1:F1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2289,7 +2741,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="70" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2341,7 +2793,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>75</v>
+        <v>85</v>
       </c>
     </row>
     <row r="6">
@@ -2351,7 +2803,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>28</v>
+        <v>35</v>
       </c>
     </row>
     <row r="7">
@@ -2361,7 +2813,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>47</v>
+        <v>50</v>
       </c>
     </row>
     <row r="8">
@@ -2371,7 +2823,19 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>10</v>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>是否达标列已新增</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
       </c>
     </row>
     <row r="10">
@@ -2380,11 +2844,7 @@
           <t>未匹配姓名</t>
         </is>
       </c>
-      <c r="B10" s="7" t="inlineStr">
-        <is>
-          <t>李胜利, 杨帆, 王玉龙, 石璇, 陆天成, 陈孟瑜, 陈晓凡, 陈海良, 韩起, 默慧宁</t>
-        </is>
-      </c>
+      <c r="B10" s="7" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
vault backup: 2026-03-25 10:19:49
</commit_message>
<xml_diff>
--- a/开发平台/codex/项目/人员简历筛选和重组/output/spreadsheet/风险项目完整清单_v1.2.xlsx
+++ b/开发平台/codex/项目/人员简历筛选和重组/output/spreadsheet/风险项目完整清单_v1.2.xlsx
@@ -462,7 +462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G88"/>
+  <dimension ref="A1:H88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -471,6 +471,7 @@
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -512,6 +513,11 @@
           <t>是否达标</t>
         </is>
       </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>所在文件夹</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="n">
@@ -538,6 +544,11 @@
           <t>否</t>
         </is>
       </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>02-风险数据加总与风险报告</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="n">
@@ -564,6 +575,11 @@
           <t>否</t>
         </is>
       </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>02-风险数据加总与风险报告</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="n">
@@ -590,6 +606,11 @@
           <t>是</t>
         </is>
       </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>02-风险数据加总与风险报告</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="n">
@@ -616,6 +637,11 @@
           <t>是</t>
         </is>
       </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>02-风险数据加总与风险报告</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="n">
@@ -640,6 +666,11 @@
       <c r="F8" s="5" t="inlineStr">
         <is>
           <t>是</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>03-业务连续性管理</t>
         </is>
       </c>
     </row>
@@ -668,6 +699,11 @@
           <t>否</t>
         </is>
       </c>
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t>03-业务连续性管理</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="n">
@@ -694,6 +730,11 @@
           <t>是</t>
         </is>
       </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>03-业务连续性管理</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="n">
@@ -720,6 +761,11 @@
           <t>是</t>
         </is>
       </c>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>03-业务连续性管理</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="n">
@@ -746,6 +792,11 @@
           <t>否</t>
         </is>
       </c>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>03-业务连续性管理</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="n">
@@ -772,6 +823,11 @@
           <t>否</t>
         </is>
       </c>
+      <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t>04-信息科技风险管理</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="n">
@@ -798,6 +854,11 @@
           <t>是</t>
         </is>
       </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>04-信息科技风险管理</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="n">
@@ -824,6 +885,11 @@
           <t>否</t>
         </is>
       </c>
+      <c r="G15" s="5" t="inlineStr">
+        <is>
+          <t>04-信息科技风险管理</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="n">
@@ -850,6 +916,11 @@
           <t>否</t>
         </is>
       </c>
+      <c r="G16" s="5" t="inlineStr">
+        <is>
+          <t>04-信息科技风险管理</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="n">
@@ -876,6 +947,11 @@
           <t>否</t>
         </is>
       </c>
+      <c r="G17" s="5" t="inlineStr">
+        <is>
+          <t>05-风险偏好与内部风险报告</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="n">
@@ -902,6 +978,11 @@
           <t>否</t>
         </is>
       </c>
+      <c r="G18" s="5" t="inlineStr">
+        <is>
+          <t>05-风险偏好与内部风险报告</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="n">
@@ -928,6 +1009,11 @@
           <t>是</t>
         </is>
       </c>
+      <c r="G19" s="5" t="inlineStr">
+        <is>
+          <t>05-风险偏好与内部风险报告</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="n">
@@ -954,6 +1040,11 @@
           <t>否</t>
         </is>
       </c>
+      <c r="G20" s="5" t="inlineStr">
+        <is>
+          <t>05-风险偏好与内部风险报告</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="n">
@@ -980,6 +1071,11 @@
           <t>否</t>
         </is>
       </c>
+      <c r="G21" s="5" t="inlineStr">
+        <is>
+          <t>05-风险偏好与内部风险报告</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="n">
@@ -1006,6 +1102,11 @@
           <t>否</t>
         </is>
       </c>
+      <c r="G22" s="5" t="inlineStr">
+        <is>
+          <t>08-分支机构和子公司风险管理能力评价</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="n">
@@ -1032,6 +1133,11 @@
           <t>否</t>
         </is>
       </c>
+      <c r="G23" s="5" t="inlineStr">
+        <is>
+          <t>08-分支机构和子公司风险管理能力评价</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="n">
@@ -1058,6 +1164,11 @@
           <t>否</t>
         </is>
       </c>
+      <c r="G24" s="5" t="inlineStr">
+        <is>
+          <t>08-分支机构和子公司风险管理能力评价</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="n">
@@ -1084,6 +1195,11 @@
           <t>是</t>
         </is>
       </c>
+      <c r="G25" s="5" t="inlineStr">
+        <is>
+          <t>08-分支机构和子公司风险管理能力评价</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="n">
@@ -1110,6 +1226,11 @@
           <t>是</t>
         </is>
       </c>
+      <c r="G26" s="5" t="inlineStr">
+        <is>
+          <t>08-分支机构和子公司风险管理能力评价</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="n">
@@ -1136,6 +1257,11 @@
           <t>是</t>
         </is>
       </c>
+      <c r="G27" s="5" t="inlineStr">
+        <is>
+          <t>09-并表管理</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="n">
@@ -1162,6 +1288,11 @@
           <t>否</t>
         </is>
       </c>
+      <c r="G28" s="5" t="inlineStr">
+        <is>
+          <t>09-并表管理</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="n">
@@ -1188,6 +1319,11 @@
           <t>否</t>
         </is>
       </c>
+      <c r="G29" s="5" t="inlineStr">
+        <is>
+          <t>09-并表管理</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="3" t="n">
@@ -1214,6 +1350,11 @@
           <t>否</t>
         </is>
       </c>
+      <c r="G30" s="5" t="inlineStr">
+        <is>
+          <t>09-并表管理</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="n">
@@ -1240,6 +1381,11 @@
           <t>是</t>
         </is>
       </c>
+      <c r="G31" s="5" t="inlineStr">
+        <is>
+          <t>09-并表管理</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="3" t="n">
@@ -1266,6 +1412,11 @@
           <t>否</t>
         </is>
       </c>
+      <c r="G32" s="5" t="inlineStr">
+        <is>
+          <t>09-并表管理</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="n">
@@ -1292,6 +1443,11 @@
           <t>是</t>
         </is>
       </c>
+      <c r="G33" s="5" t="inlineStr">
+        <is>
+          <t>10-限额管理</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="3" t="n">
@@ -1318,6 +1474,11 @@
           <t>否</t>
         </is>
       </c>
+      <c r="G34" s="5" t="inlineStr">
+        <is>
+          <t>10-限额管理</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="n">
@@ -1344,6 +1505,11 @@
           <t>否</t>
         </is>
       </c>
+      <c r="G35" s="5" t="inlineStr">
+        <is>
+          <t>10-限额管理</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="3" t="n">
@@ -1370,6 +1536,11 @@
           <t>是</t>
         </is>
       </c>
+      <c r="G36" s="5" t="inlineStr">
+        <is>
+          <t>10-限额管理</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="3" t="n">
@@ -1396,6 +1567,11 @@
           <t>否</t>
         </is>
       </c>
+      <c r="G37" s="5" t="inlineStr">
+        <is>
+          <t>10-限额管理</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="3" t="n">
@@ -1422,6 +1598,11 @@
           <t>否</t>
         </is>
       </c>
+      <c r="G38" s="5" t="inlineStr">
+        <is>
+          <t>11-压力测试</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="3" t="n">
@@ -1448,6 +1629,11 @@
           <t>否</t>
         </is>
       </c>
+      <c r="G39" s="5" t="inlineStr">
+        <is>
+          <t>11-压力测试</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="3" t="n">
@@ -1474,6 +1660,11 @@
           <t>否</t>
         </is>
       </c>
+      <c r="G40" s="5" t="inlineStr">
+        <is>
+          <t>11-压力测试</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="3" t="n">
@@ -1500,6 +1691,11 @@
           <t>否</t>
         </is>
       </c>
+      <c r="G41" s="5" t="inlineStr">
+        <is>
+          <t>11-压力测试</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="3" t="n">
@@ -1526,6 +1722,11 @@
           <t>是</t>
         </is>
       </c>
+      <c r="G42" s="5" t="inlineStr">
+        <is>
+          <t>11-压力测试</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="3" t="n">
@@ -1552,6 +1753,11 @@
           <t>是</t>
         </is>
       </c>
+      <c r="G43" s="5" t="inlineStr">
+        <is>
+          <t>13-模型管理</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="3" t="n">
@@ -1578,6 +1784,11 @@
           <t>是</t>
         </is>
       </c>
+      <c r="G44" s="5" t="inlineStr">
+        <is>
+          <t>13-模型管理</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="3" t="n">
@@ -1604,6 +1815,11 @@
           <t>否</t>
         </is>
       </c>
+      <c r="G45" s="5" t="inlineStr">
+        <is>
+          <t>13-模型管理</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="3" t="n">
@@ -1630,6 +1846,11 @@
           <t>否</t>
         </is>
       </c>
+      <c r="G46" s="5" t="inlineStr">
+        <is>
+          <t>13-模型管理</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="3" t="n">
@@ -1656,6 +1877,11 @@
           <t>否</t>
         </is>
       </c>
+      <c r="G47" s="5" t="inlineStr">
+        <is>
+          <t>13-模型管理</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="3" t="n">
@@ -1682,6 +1908,11 @@
           <t>否</t>
         </is>
       </c>
+      <c r="G48" s="5" t="inlineStr">
+        <is>
+          <t>14-风险提示管理</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="3" t="n">
@@ -1708,6 +1939,11 @@
           <t>是</t>
         </is>
       </c>
+      <c r="G49" s="5" t="inlineStr">
+        <is>
+          <t>14-风险提示管理</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="3" t="n">
@@ -1734,6 +1970,11 @@
           <t>是</t>
         </is>
       </c>
+      <c r="G50" s="5" t="inlineStr">
+        <is>
+          <t>14-风险提示管理</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="3" t="n">
@@ -1760,6 +2001,11 @@
           <t>否</t>
         </is>
       </c>
+      <c r="G51" s="5" t="inlineStr">
+        <is>
+          <t>14-风险提示管理</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="3" t="n">
@@ -1786,6 +2032,11 @@
           <t>否</t>
         </is>
       </c>
+      <c r="G52" s="5" t="inlineStr">
+        <is>
+          <t>14-风险提示管理</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="3" t="n">
@@ -1812,6 +2063,11 @@
           <t>是</t>
         </is>
       </c>
+      <c r="G53" s="5" t="inlineStr">
+        <is>
+          <t>14-风险提示管理</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="3" t="n">
@@ -1838,6 +2094,11 @@
           <t>否</t>
         </is>
       </c>
+      <c r="G54" s="5" t="inlineStr">
+        <is>
+          <t>15-专家团队</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="3" t="n">
@@ -1864,6 +2125,11 @@
           <t>否</t>
         </is>
       </c>
+      <c r="G55" s="5" t="inlineStr">
+        <is>
+          <t>15-专家团队</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="3" t="n">
@@ -1890,6 +2156,11 @@
           <t>否</t>
         </is>
       </c>
+      <c r="G56" s="5" t="inlineStr">
+        <is>
+          <t>15-专家团队</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="3" t="n">
@@ -1916,6 +2187,11 @@
           <t>否</t>
         </is>
       </c>
+      <c r="G57" s="5" t="inlineStr">
+        <is>
+          <t>15-专家团队</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="3" t="n">
@@ -1942,6 +2218,11 @@
           <t>否</t>
         </is>
       </c>
+      <c r="G58" s="5" t="inlineStr">
+        <is>
+          <t>15-专家团队</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="3" t="n">
@@ -1968,6 +2249,11 @@
           <t>是</t>
         </is>
       </c>
+      <c r="G59" s="5" t="inlineStr">
+        <is>
+          <t>16-常规团队</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="3" t="n">
@@ -1994,6 +2280,11 @@
           <t>是</t>
         </is>
       </c>
+      <c r="G60" s="5" t="inlineStr">
+        <is>
+          <t>16-常规团队</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="3" t="n">
@@ -2020,6 +2311,11 @@
           <t>是</t>
         </is>
       </c>
+      <c r="G61" s="5" t="inlineStr">
+        <is>
+          <t>16-常规团队</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="3" t="n">
@@ -2046,6 +2342,11 @@
           <t>是</t>
         </is>
       </c>
+      <c r="G62" s="5" t="inlineStr">
+        <is>
+          <t>16-常规团队</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="3" t="n">
@@ -2072,6 +2373,11 @@
           <t>是</t>
         </is>
       </c>
+      <c r="G63" s="5" t="inlineStr">
+        <is>
+          <t>16-常规团队</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="3" t="n">
@@ -2098,6 +2404,11 @@
           <t>是</t>
         </is>
       </c>
+      <c r="G64" s="5" t="inlineStr">
+        <is>
+          <t>16-常规团队</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="3" t="n">
@@ -2124,6 +2435,11 @@
           <t>是</t>
         </is>
       </c>
+      <c r="G65" s="5" t="inlineStr">
+        <is>
+          <t>16-常规团队</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="3" t="n">
@@ -2150,6 +2466,11 @@
           <t>是</t>
         </is>
       </c>
+      <c r="G66" s="5" t="inlineStr">
+        <is>
+          <t>企业级风险管理平台</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="3" t="n">
@@ -2176,6 +2497,11 @@
           <t>否</t>
         </is>
       </c>
+      <c r="G67" s="5" t="inlineStr">
+        <is>
+          <t>企业级风险管理平台</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="3" t="n">
@@ -2202,6 +2528,11 @@
           <t>否</t>
         </is>
       </c>
+      <c r="G68" s="5" t="inlineStr">
+        <is>
+          <t>企业级风险管理平台</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="3" t="n">
@@ -2228,6 +2559,11 @@
           <t>否</t>
         </is>
       </c>
+      <c r="G69" s="5" t="inlineStr">
+        <is>
+          <t>企业级风险管理平台</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="3" t="n">
@@ -2254,6 +2590,11 @@
           <t>是</t>
         </is>
       </c>
+      <c r="G70" s="5" t="inlineStr">
+        <is>
+          <t>企业级风险管理平台</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="3" t="n">
@@ -2280,6 +2621,11 @@
           <t>否</t>
         </is>
       </c>
+      <c r="G71" s="5" t="inlineStr">
+        <is>
+          <t>企业级风险管理平台</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="3" t="n">
@@ -2306,6 +2652,11 @@
           <t>否</t>
         </is>
       </c>
+      <c r="G72" s="5" t="inlineStr">
+        <is>
+          <t>企业级风险管理平台</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="3" t="n">
@@ -2332,6 +2683,11 @@
           <t>否</t>
         </is>
       </c>
+      <c r="G73" s="5" t="inlineStr">
+        <is>
+          <t>企业级风险管理平台</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="3" t="n">
@@ -2358,6 +2714,11 @@
           <t>是</t>
         </is>
       </c>
+      <c r="G74" s="5" t="inlineStr">
+        <is>
+          <t>企业级风险管理平台</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="3" t="n">
@@ -2384,6 +2745,11 @@
           <t>否</t>
         </is>
       </c>
+      <c r="G75" s="5" t="inlineStr">
+        <is>
+          <t>后评价工作</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="3" t="n">
@@ -2410,6 +2776,11 @@
           <t>否</t>
         </is>
       </c>
+      <c r="G76" s="5" t="inlineStr">
+        <is>
+          <t>后评价工作</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="3" t="n">
@@ -2436,6 +2807,11 @@
           <t>否</t>
         </is>
       </c>
+      <c r="G77" s="5" t="inlineStr">
+        <is>
+          <t>后评价工作</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="3" t="n">
@@ -2462,6 +2838,11 @@
           <t>是</t>
         </is>
       </c>
+      <c r="G78" s="5" t="inlineStr">
+        <is>
+          <t>后评价工作</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="3" t="n">
@@ -2488,6 +2869,11 @@
           <t>否</t>
         </is>
       </c>
+      <c r="G79" s="5" t="inlineStr">
+        <is>
+          <t>后评价工作</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="3" t="n">
@@ -2514,6 +2900,11 @@
           <t>是</t>
         </is>
       </c>
+      <c r="G80" s="5" t="inlineStr">
+        <is>
+          <t>恢复与处置计划管理</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="3" t="n">
@@ -2540,6 +2931,11 @@
           <t>否</t>
         </is>
       </c>
+      <c r="G81" s="5" t="inlineStr">
+        <is>
+          <t>恢复与处置计划管理</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="3" t="n">
@@ -2566,6 +2962,11 @@
           <t>否</t>
         </is>
       </c>
+      <c r="G82" s="5" t="inlineStr">
+        <is>
+          <t>恢复与处置计划管理</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="3" t="n">
@@ -2592,6 +2993,11 @@
           <t>是</t>
         </is>
       </c>
+      <c r="G83" s="5" t="inlineStr">
+        <is>
+          <t>恢复与处置计划管理</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="3" t="n">
@@ -2618,6 +3024,11 @@
           <t>是</t>
         </is>
       </c>
+      <c r="G84" s="5" t="inlineStr">
+        <is>
+          <t>恢复与处置计划管理</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="3" t="n">
@@ -2644,6 +3055,11 @@
           <t>否</t>
         </is>
       </c>
+      <c r="G85" s="5" t="inlineStr">
+        <is>
+          <t>风险文化</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="3" t="n">
@@ -2670,6 +3086,11 @@
           <t>是</t>
         </is>
       </c>
+      <c r="G86" s="5" t="inlineStr">
+        <is>
+          <t>风险文化</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="3" t="n">
@@ -2696,6 +3117,11 @@
           <t>是</t>
         </is>
       </c>
+      <c r="G87" s="5" t="inlineStr">
+        <is>
+          <t>风险文化</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="3" t="n">
@@ -2722,10 +3148,15 @@
           <t>否</t>
         </is>
       </c>
+      <c r="G88" s="5" t="inlineStr">
+        <is>
+          <t>风险文化</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A1:G1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>